<commit_message>
Re-add documents and additional refactors for pipeline
</commit_message>
<xml_diff>
--- a/thesis/pipeline/result/evaluation/requirement/design/v1/CF_M01/CF_M01_req_eval_avg_by_type.xlsx
+++ b/thesis/pipeline/result/evaluation/requirement/design/v1/CF_M01/CF_M01_req_eval_avg_by_type.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>recall</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>f1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -485,6 +490,9 @@
       <c r="H2" t="n">
         <v>0.7059</v>
       </c>
+      <c r="I2" t="n">
+        <v>0.8276</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -513,6 +521,9 @@
       <c r="H3" t="n">
         <v>1</v>
       </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -541,6 +552,9 @@
       <c r="H4" t="n">
         <v>0.6667</v>
       </c>
+      <c r="I4" t="n">
+        <v>0.6667</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -568,6 +582,9 @@
       </c>
       <c r="H5" t="n">
         <v>0.3333</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>